<commit_message>
feat: 장비 분해 재료 표 DisassembleTable을 만든다 (T-131)
</commit_message>
<xml_diff>
--- a/GameDesign/Excel/Equip.xlsx
+++ b/GameDesign/Excel/Equip.xlsx
@@ -7,6 +7,7 @@
   </bookViews>
   <sheets>
     <sheet name="EquipTable" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="DisassembleTable" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="0" fullCalcOnLoad="1"/>
@@ -117,7 +118,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -156,6 +157,12 @@
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -3497,4 +3504,306 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="15" customWidth="1" min="1" max="1"/>
+    <col width="15" customWidth="1" min="2" max="2"/>
+    <col width="19" customWidth="1" min="3" max="3"/>
+    <col width="11" customWidth="1" min="4" max="4"/>
+    <col width="36" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="8" t="n"/>
+      <c r="B1" s="8" t="n"/>
+      <c r="C1" s="8" t="n"/>
+      <c r="D1" s="8" t="n"/>
+      <c r="E1" s="8" t="n"/>
+    </row>
+    <row r="2">
+      <c r="A2" s="9" t="inlineStr">
+        <is>
+          <t>//</t>
+        </is>
+      </c>
+      <c r="B2" s="10" t="inlineStr">
+        <is>
+          <t>등급</t>
+        </is>
+      </c>
+      <c r="C2" s="10" t="inlineStr">
+        <is>
+          <t>재료</t>
+        </is>
+      </c>
+      <c r="D2" s="10" t="inlineStr">
+        <is>
+          <t>수량</t>
+        </is>
+      </c>
+      <c r="E2" s="10" t="inlineStr">
+        <is>
+          <t>메모</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="9" t="inlineStr">
+        <is>
+          <t>C&amp;S</t>
+        </is>
+      </c>
+      <c r="B3" s="11" t="inlineStr">
+        <is>
+          <t>a</t>
+        </is>
+      </c>
+      <c r="C3" s="11" t="inlineStr">
+        <is>
+          <t>a</t>
+        </is>
+      </c>
+      <c r="D3" s="11" t="inlineStr">
+        <is>
+          <t>a</t>
+        </is>
+      </c>
+      <c r="E3" s="11" t="inlineStr">
+        <is>
+          <t>a</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="9" t="inlineStr">
+        <is>
+          <t>Type</t>
+        </is>
+      </c>
+      <c r="B4" s="11" t="inlineStr">
+        <is>
+          <t>eGlobalRarity</t>
+        </is>
+      </c>
+      <c r="C4" s="11" t="inlineStr">
+        <is>
+          <t>int</t>
+        </is>
+      </c>
+      <c r="D4" s="11" t="inlineStr">
+        <is>
+          <t>int</t>
+        </is>
+      </c>
+      <c r="E4" s="11" t="inlineStr">
+        <is>
+          <t>string</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="9" t="inlineStr">
+        <is>
+          <t>Min</t>
+        </is>
+      </c>
+      <c r="B5" s="11" t="n"/>
+      <c r="C5" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="D5" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="E5" s="11" t="n"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="9" t="inlineStr">
+        <is>
+          <t>Max</t>
+        </is>
+      </c>
+      <c r="B6" s="11" t="n"/>
+      <c r="C6" s="11" t="n"/>
+      <c r="D6" s="11" t="n"/>
+      <c r="E6" s="11" t="n"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="9" t="inlineStr">
+        <is>
+          <t>Default(Null)</t>
+        </is>
+      </c>
+      <c r="B7" s="11" t="n"/>
+      <c r="C7" s="11" t="n"/>
+      <c r="D7" s="11" t="n"/>
+      <c r="E7" s="11" t="inlineStr">
+        <is>
+          <t>""</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="9" t="inlineStr">
+        <is>
+          <t>Ref</t>
+        </is>
+      </c>
+      <c r="B8" s="11" t="n"/>
+      <c r="C8" s="11" t="inlineStr">
+        <is>
+          <t>ItemTable.ItemTID</t>
+        </is>
+      </c>
+      <c r="D8" s="11" t="n"/>
+      <c r="E8" s="11" t="n"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="8" t="n"/>
+      <c r="B9" s="12" t="inlineStr">
+        <is>
+          <t>Rarity</t>
+        </is>
+      </c>
+      <c r="C9" s="12" t="inlineStr">
+        <is>
+          <t>ItemTID</t>
+        </is>
+      </c>
+      <c r="D9" s="12" t="inlineStr">
+        <is>
+          <t>ItemCount</t>
+        </is>
+      </c>
+      <c r="E9" s="12" t="inlineStr">
+        <is>
+          <t>Description</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="8" t="n"/>
+      <c r="B10" s="15" t="inlineStr">
+        <is>
+          <t>Common</t>
+        </is>
+      </c>
+      <c r="C10" s="16" t="n">
+        <v>100050</v>
+      </c>
+      <c r="D10" s="16" t="n">
+        <v>1</v>
+      </c>
+      <c r="E10" s="15" t="inlineStr">
+        <is>
+          <t>일반 장비 분해 → 마력의 파편 1개</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="8" t="n"/>
+      <c r="B11" s="15" t="inlineStr">
+        <is>
+          <t>Uncommon</t>
+        </is>
+      </c>
+      <c r="C11" s="16" t="n">
+        <v>100050</v>
+      </c>
+      <c r="D11" s="16" t="n">
+        <v>2</v>
+      </c>
+      <c r="E11" s="15" t="inlineStr">
+        <is>
+          <t>고급 장비 분해 → 마력의 파편 2개</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="8" t="n"/>
+      <c r="B12" s="15" t="inlineStr">
+        <is>
+          <t>Rare</t>
+        </is>
+      </c>
+      <c r="C12" s="16" t="n">
+        <v>100050</v>
+      </c>
+      <c r="D12" s="16" t="n">
+        <v>5</v>
+      </c>
+      <c r="E12" s="15" t="inlineStr">
+        <is>
+          <t>희귀 장비 분해 → 마력의 파편 5개</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="8" t="n"/>
+      <c r="B13" s="15" t="inlineStr">
+        <is>
+          <t>Epic</t>
+        </is>
+      </c>
+      <c r="C13" s="16" t="n">
+        <v>100050</v>
+      </c>
+      <c r="D13" s="16" t="n">
+        <v>15</v>
+      </c>
+      <c r="E13" s="15" t="inlineStr">
+        <is>
+          <t>영웅 장비 분해 → 마력의 파편 15개</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="8" t="n"/>
+      <c r="B14" s="15" t="inlineStr">
+        <is>
+          <t>Legendary</t>
+        </is>
+      </c>
+      <c r="C14" s="16" t="n">
+        <v>100050</v>
+      </c>
+      <c r="D14" s="16" t="n">
+        <v>50</v>
+      </c>
+      <c r="E14" s="15" t="inlineStr">
+        <is>
+          <t>전설 장비 분해 → 마력의 파편 50개</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="8" t="n"/>
+      <c r="B15" s="15" t="inlineStr">
+        <is>
+          <t>Mythic</t>
+        </is>
+      </c>
+      <c r="C15" s="16" t="n">
+        <v>100050</v>
+      </c>
+      <c r="D15" s="16" t="n">
+        <v>150</v>
+      </c>
+      <c r="E15" s="15" t="inlineStr">
+        <is>
+          <t>신화 장비 분해 → 마력의 파편 150개</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>